<commit_message>
Add Question Scoring sheet with pairwise relevance matrix
Scores each of the 18 consolidated questions against every other question
(1-5) for thematic/content overlap, to surface residual redundancy beyond
what was merged into the Consolidated sheet. Includes a legend, question
key, color-coded 18x18 matrix, per-question averages, and a shortlist of
notable overlaps (score 4-5) with rationale. Consolidated and Draft Master
Question sheets are unchanged.
</commit_message>
<xml_diff>
--- a/deliverables/Survey_Question_Master_List.xlsx
+++ b/deliverables/Survey_Question_Master_List.xlsx
@@ -7,7 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="Consolidated" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Draft Master Question" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Question Scoring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Draft Master Question" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +45,21 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00006B6B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +85,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E6F4F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -167,6 +186,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1179,6 +1212,2084 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:T69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Relevance / overlap scoring legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Most relevant — near-duplicate; same construct, likely redundant data</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Relevant — same theme, closely related angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Same relevancy — same broad category, distinct angle/sub-topic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Less relevant — different themes, loosely related</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Very less relevant — essentially unrelated themes/constructs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Question key</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Q-ID</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Clarity &amp; Awareness</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>How clear is your career development pathway within Gentari for your current role (tech...</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Clarity &amp; Awareness</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>Are you aware of any structured training or development programs available for your gro...</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Clarity &amp; Awareness</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Do you feel the expectations and criteria for promotion in your role are clearly defined?</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Effectiveness &amp; Adequacy of Development Support</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>How would you rate both the accessibility and adequacy of learning and development reso...</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Effectiveness of Existing Programs</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>How fairly and consistently are promotion and growth opportunities applied across teams...</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Expectations &amp; Improvement Areas</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>If Gentari could improve one aspect of career development, which would create the great...</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Expectations &amp; Improvement Areas</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Would you prefer a more clearly defined career path framework (technical vs managerial ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Career Growth Challenges</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>Which of the following best describes the biggest challenge you face in developing your...</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Future-Readiness &amp; Skill Obsolescence</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>How confident are you that the development support available within Gentari is keeping ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Stretch Assignments &amp; Technical Exposure</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>How frequently are you given the opportunity to work on projects or assignments outside...</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Individual Development Plan (IDP)</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Do you currently have a formal Individual Development Plan (IDP) agreed with your manag...</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Gauging Severity of the Issue</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>To what extent does this challenge impact your motivation and performance at work? (as ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Root Cause Perception</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>What do you believe is the primary reason for this issue?</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Retention</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>Do you see yourself still being within the business in the next 12 months?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>From a talent growth and retention perspective, is there anything you would like to tel...</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>2030 EBITDA Target Awareness</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>How aware are you of Gentari's aspiration to achieve an EBITDA of US$613 million by 2030?</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>2030 EBITDA Target Awareness</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>How well do you understand your role and team's contribution towards achieving the 2030...</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2030 EBITDA Target Awareness</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>In your opinion, what are the biggest barriers that could prevent Gentari from achievin...</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Pairwise relevance matrix (1-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr"/>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="L30" s="17" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="M30" s="17" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="N30" s="17" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="O30" s="17" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="P30" s="17" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="Q30" s="17" t="inlineStr">
+        <is>
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="R30" s="17" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="S30" s="17" t="inlineStr">
+        <is>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="T30" s="17" t="inlineStr">
+        <is>
+          <t>Avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I31" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T31" s="20" t="n">
+        <v>2.06</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T32" s="20" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="I33" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T33" s="20" t="n">
+        <v>2.12</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="K34" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L34" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="O34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S34" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T34" s="20" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I35" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T35" s="20" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I36" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="J36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L36" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M36" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="N36" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="O36" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q36" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R36" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T36" s="20" t="n">
+        <v>2.29</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N37" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="O37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P37" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T37" s="20" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="H38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="N38" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="O38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P38" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T38" s="20" t="n">
+        <v>2.59</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J39" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="L39" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T39" s="20" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="K40" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S40" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T40" s="20" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J41" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="K41" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L41" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P41" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T41" s="20" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N42" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="O42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P42" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T42" s="20" t="n">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H43" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I43" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J43" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="N43" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P43" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T43" s="20" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O44" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P44" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="R44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S44" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="T44" s="20" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="H45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="I45" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J45" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="N45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="O45" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="P45" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="R45" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="S45" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="T45" s="20" t="n">
+        <v>2.24</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O46" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P46" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q46" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R46" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="S46" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="T46" s="20" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O47" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P47" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q47" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="R47" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S47" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="T47" s="20" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="O48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P48" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q48" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="R48" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="S48" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T48" s="20" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>Avg</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="C49" s="20" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="D49" s="20" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="E49" s="20" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="F49" s="20" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="G49" s="20" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="H49" s="20" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="I49" s="20" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="J49" s="20" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="K49" s="20" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="L49" s="20" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="M49" s="20" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="N49" s="20" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="O49" s="20" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="P49" s="20" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="Q49" s="20" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="R49" s="20" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="S49" s="20" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>Notable overlaps (score 4-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Pair</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>Q1 &lt;-&gt; Q7</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>Near-duplicate: both ask about having a clearly defined career-path structure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>Q3 &lt;-&gt; Q5</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Both are about how promotion decisions are made (clarity vs. fairness/consistency).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t>Q6 &lt;-&gt; Q8</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>Two sides of the same coin: desired fix vs. the pain point it would fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>Q8 &lt;-&gt; Q12</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Q12 is an explicit follow-up to the biggest-challenge question (Q8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>Q16 &lt;-&gt; Q17</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>Both measure awareness/understanding of the 2030 EBITDA target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>Q1 &lt;-&gt; Q3</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>Both measure clarity of the advancement structure (path vs. promotion criteria).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>Q2 &lt;-&gt; Q4</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>Both concern availability/quality of the same L&amp;D resources (awareness vs. accessibility &amp; adequacy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="14" t="inlineStr">
+        <is>
+          <t>Q3 &lt;-&gt; Q7</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" s="14" t="inlineStr">
+        <is>
+          <t>Both about structural clarity of career advancement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="inlineStr">
+        <is>
+          <t>Q3 &lt;-&gt; Q8</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>The challenge MCQ explicitly includes 'promotion criteria are unclear' as an option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>Q4 &lt;-&gt; Q9</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>Both measure sufficiency of development support (general adequacy vs. technical skill currency).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>Q6 &lt;-&gt; Q15</t>
+        </is>
+      </c>
+      <c r="B63" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>Same intent (what would help), different format: closed MCQ vs. open catch-all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>Q8 &lt;-&gt; Q13</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>Root cause is asked about the same 'issue' identified by the challenge question (Q8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>Q9 &lt;-&gt; Q10</t>
+        </is>
+      </c>
+      <c r="B65" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" s="12" t="inlineStr">
+        <is>
+          <t>Both are Ungku's technical-exposure sub-questions (skill currency vs. stretch assignments).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>Q12 &lt;-&gt; Q13</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>Paired diagnostic questions about the same issue: severity and root cause.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>Q14 &lt;-&gt; Q15</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C67" s="12" t="inlineStr">
+        <is>
+          <t>Mark Turner's retention/development pair — both about staying/leaving sentiment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="inlineStr">
+        <is>
+          <t>Q16 &lt;-&gt; Q18</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>Same EBITDA-target topic cluster (awareness vs. barriers).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>Q17 &lt;-&gt; Q18</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" s="12" t="inlineStr">
+        <is>
+          <t>Same EBITDA-target topic cluster (role contribution vs. barriers).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B31:S48">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="3"/>
+        <cfvo type="num" val="5"/>
+        <color rgb="00C6EFCE"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>

</xml_diff>

<commit_message>
Make Question Scoring matrix directional with live Sum/Priority formulas
Cell (row Qi, col Qj) is now "from Qi's point of view, how relevant is
Qj" (1-5); only cells where row Q# < column Q# are independently judged,
the mirrored cell is a live formula (reverse = 6 - forward). Replaces the
Avg row/column with a Sum column (formula-based, adds only the
independently-judged values touching each question so a question's
position in the Q1-Q18 list doesn't skew it) and a Priority column
(=RANK on Sum, descending). Notable-overlaps list relabeled as
directional. Consolidated and Draft Master Question sheets unchanged.
</commit_message>
<xml_diff>
--- a/deliverables/Survey_Question_Master_List.xlsx
+++ b/deliverables/Survey_Question_Master_List.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -145,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -201,6 +205,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1212,35 +1217,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T69"/>
+  <dimension ref="A1:U69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
-    <col width="7" customWidth="1" min="18" max="18"/>
-    <col width="7" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="9" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Relevance / overlap scoring legend</t>
+          <t>Relevance scoring legend</t>
         </is>
       </c>
     </row>
@@ -1304,538 +1310,490 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>How to read a cell:</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Each cell = "from the ROW question's point of view, how relevant is the COLUMN question" (1-5). Only cells where the row's Q-number is smaller than the column's Q-number were independently judged; the mirrored cell (row Q-number &gt; column Q-number) is a live formula: reverse = 6 - forward.
+Sum/Priority: Sum adds up only the independently-judged values touching a question (not a plain row total) so a question's position in the Q1-Q18 list doesn't skew its score. Priority = rank of Sum, descending (1 = most relevant to the rest of the set overall = top priority to review).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Question key</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Q-ID</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Theme</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Clarity &amp; Awareness</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>How clear is your career development pathway within Gentari for your current role (tech...</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Clarity &amp; Awareness</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Are you aware of any structured training or development programs available for your gro...</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Clarity &amp; Awareness</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Do you feel the expectations and criteria for promotion in your role are clearly defined?</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Effectiveness &amp; Adequacy of Development Support</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>How would you rate both the accessibility and adequacy of learning and development reso...</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Q5</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Effectiveness of Existing Programs</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>How fairly and consistently are promotion and growth opportunities applied across teams...</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Expectations &amp; Improvement Areas</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>If Gentari could improve one aspect of career development, which would create the great...</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Q7</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Expectations &amp; Improvement Areas</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Would you prefer a more clearly defined career path framework (technical vs managerial ...</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Career Growth Challenges</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Which of the following best describes the biggest challenge you face in developing your...</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Q9</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Future-Readiness &amp; Skill Obsolescence</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>How confident are you that the development support available within Gentari is keeping ...</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Q10</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Stretch Assignments &amp; Technical Exposure</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>How frequently are you given the opportunity to work on projects or assignments outside...</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Q11</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Individual Development Plan (IDP)</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C21" s="12" t="inlineStr">
         <is>
           <t>Do you currently have a formal Individual Development Plan (IDP) agreed with your manag...</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Q12</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Gauging Severity of the Issue</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>To what extent does this challenge impact your motivation and performance at work? (as ...</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Q13</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Root Cause Perception</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C23" s="12" t="inlineStr">
         <is>
           <t>What do you believe is the primary reason for this issue?</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Q14</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Retention</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>Do you see yourself still being within the business in the next 12 months?</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Q15</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Development</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>From a talent growth and retention perspective, is there anything you would like to tel...</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Q16</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>2030 EBITDA Target Awareness</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>How aware are you of Gentari's aspiration to achieve an EBITDA of US$613 million by 2030?</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Q17</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>2030 EBITDA Target Awareness</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>How well do you understand your role and team's contribution towards achieving the 2030...</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Q18</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>2030 EBITDA Target Awareness</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>In your opinion, what are the biggest barriers that could prevent Gentari from achievin...</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>Pairwise relevance matrix (1-5)</t>
-        </is>
-      </c>
-    </row>
     <row r="30">
-      <c r="A30" s="17" t="inlineStr"/>
-      <c r="B30" s="17" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Directional relevance matrix (1-5): row -&gt; column</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr"/>
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
       </c>
-      <c r="C30" s="17" t="inlineStr">
+      <c r="C31" s="17" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
-      <c r="D30" s="17" t="inlineStr">
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
       </c>
-      <c r="E30" s="17" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
       </c>
-      <c r="F30" s="17" t="inlineStr">
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>Q5</t>
         </is>
       </c>
-      <c r="G30" s="17" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="H30" s="17" t="inlineStr">
+      <c r="H31" s="17" t="inlineStr">
         <is>
           <t>Q7</t>
         </is>
       </c>
-      <c r="I30" s="17" t="inlineStr">
+      <c r="I31" s="17" t="inlineStr">
         <is>
           <t>Q8</t>
         </is>
       </c>
-      <c r="J30" s="17" t="inlineStr">
+      <c r="J31" s="17" t="inlineStr">
         <is>
           <t>Q9</t>
         </is>
       </c>
-      <c r="K30" s="17" t="inlineStr">
+      <c r="K31" s="17" t="inlineStr">
         <is>
           <t>Q10</t>
         </is>
       </c>
-      <c r="L30" s="17" t="inlineStr">
+      <c r="L31" s="17" t="inlineStr">
         <is>
           <t>Q11</t>
         </is>
       </c>
-      <c r="M30" s="17" t="inlineStr">
+      <c r="M31" s="17" t="inlineStr">
         <is>
           <t>Q12</t>
         </is>
       </c>
-      <c r="N30" s="17" t="inlineStr">
+      <c r="N31" s="17" t="inlineStr">
         <is>
           <t>Q13</t>
         </is>
       </c>
-      <c r="O30" s="17" t="inlineStr">
+      <c r="O31" s="17" t="inlineStr">
         <is>
           <t>Q14</t>
         </is>
       </c>
-      <c r="P30" s="17" t="inlineStr">
+      <c r="P31" s="17" t="inlineStr">
         <is>
           <t>Q15</t>
         </is>
       </c>
-      <c r="Q30" s="17" t="inlineStr">
+      <c r="Q31" s="17" t="inlineStr">
         <is>
           <t>Q16</t>
         </is>
       </c>
-      <c r="R30" s="17" t="inlineStr">
+      <c r="R31" s="17" t="inlineStr">
         <is>
           <t>Q17</t>
         </is>
       </c>
-      <c r="S30" s="17" t="inlineStr">
+      <c r="S31" s="17" t="inlineStr">
         <is>
           <t>Q18</t>
         </is>
       </c>
-      <c r="T30" s="17" t="inlineStr">
-        <is>
-          <t>Avg</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="B31" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C31" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="D31" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="E31" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F31" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="G31" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="I31" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="J31" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="M31" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N31" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O31" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P31" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q31" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="R31" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="S31" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="T31" s="20" t="n">
-        <v>2.06</v>
+      <c r="T31" s="17" t="inlineStr">
+        <is>
+          <t>Sum</t>
+        </is>
+      </c>
+      <c r="U31" s="17" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="B32" s="19" t="n">
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="D32" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="E32" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="F32" s="19" t="n">
-        <v>2</v>
-      </c>
       <c r="G32" s="19" t="n">
         <v>2</v>
       </c>
       <c r="H32" s="19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I32" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J32" s="19" t="n">
         <v>2</v>
@@ -1867,50 +1825,56 @@
       <c r="S32" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T32" s="20" t="n">
-        <v>1.88</v>
+      <c r="T32" s="20">
+        <f>SUM(C32:S32)</f>
+        <v/>
+      </c>
+      <c r="U32" s="20">
+        <f>RANK(T32,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="n">
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B33" s="19">
+        <f>6-C32</f>
+        <v/>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="F33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="D33" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E33" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="G33" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="I33" s="19" t="n">
-        <v>4</v>
-      </c>
       <c r="J33" s="19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33" s="19" t="n">
         <v>1</v>
       </c>
       <c r="L33" s="19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M33" s="19" t="n">
         <v>1</v>
@@ -1933,56 +1897,63 @@
       <c r="S33" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T33" s="20" t="n">
-        <v>2.12</v>
+      <c r="T33" s="20">
+        <f>SUM(D33:S33)+SUM(C32:C32)</f>
+        <v/>
+      </c>
+      <c r="U33" s="20">
+        <f>RANK(T33,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="B34" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C34" s="19" t="n">
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B34" s="19">
+        <f>6-D32</f>
+        <v/>
+      </c>
+      <c r="C34" s="19">
+        <f>6-D33</f>
+        <v/>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F34" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="G34" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="H34" s="19" t="n">
-        <v>1</v>
-      </c>
       <c r="I34" s="19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J34" s="19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K34" s="19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L34" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M34" s="19" t="n">
         <v>1</v>
       </c>
       <c r="N34" s="19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O34" s="19" t="n">
         <v>1</v>
@@ -1999,56 +1970,64 @@
       <c r="S34" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T34" s="20" t="n">
-        <v>2.18</v>
+      <c r="T34" s="20">
+        <f>SUM(E34:S34)+SUM(D32:D33)</f>
+        <v/>
+      </c>
+      <c r="U34" s="20">
+        <f>RANK(T34,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>Q5</t>
-        </is>
-      </c>
-      <c r="B35" s="19" t="n">
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B35" s="19">
+        <f>6-E32</f>
+        <v/>
+      </c>
+      <c r="C35" s="19">
+        <f>6-E33</f>
+        <v/>
+      </c>
+      <c r="D35" s="19">
+        <f>6-E34</f>
+        <v/>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C35" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="E35" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="19" t="n">
-        <v>2</v>
-      </c>
       <c r="H35" s="19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I35" s="19" t="n">
         <v>3</v>
       </c>
       <c r="J35" s="19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K35" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L35" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M35" s="19" t="n">
         <v>1</v>
       </c>
       <c r="N35" s="19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O35" s="19" t="n">
         <v>1</v>
@@ -2065,62 +2044,71 @@
       <c r="S35" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T35" s="20" t="n">
-        <v>1.88</v>
+      <c r="T35" s="20">
+        <f>SUM(F35:S35)+SUM(E32:E34)</f>
+        <v/>
+      </c>
+      <c r="U35" s="20">
+        <f>RANK(T35,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="B36" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C36" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D36" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F36" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" s="18" t="inlineStr">
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="B36" s="19">
+        <f>6-F32</f>
+        <v/>
+      </c>
+      <c r="C36" s="19">
+        <f>6-F33</f>
+        <v/>
+      </c>
+      <c r="D36" s="19">
+        <f>6-F34</f>
+        <v/>
+      </c>
+      <c r="E36" s="19">
+        <f>6-F35</f>
+        <v/>
+      </c>
+      <c r="F36" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="G36" s="19" t="n">
+        <v>2</v>
       </c>
       <c r="H36" s="19" t="n">
         <v>3</v>
       </c>
       <c r="I36" s="19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J36" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K36" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L36" s="19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M36" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N36" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O36" s="19" t="n">
         <v>1</v>
       </c>
       <c r="P36" s="19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q36" s="19" t="n">
         <v>1</v>
@@ -2131,53 +2119,63 @@
       <c r="S36" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T36" s="20" t="n">
-        <v>2.29</v>
+      <c r="T36" s="20">
+        <f>SUM(G36:S36)+SUM(F32:F35)</f>
+        <v/>
+      </c>
+      <c r="U36" s="20">
+        <f>RANK(T36,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>Q7</t>
-        </is>
-      </c>
-      <c r="B37" s="19" t="n">
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="B37" s="19">
+        <f>6-G32</f>
+        <v/>
+      </c>
+      <c r="C37" s="19">
+        <f>6-G33</f>
+        <v/>
+      </c>
+      <c r="D37" s="19">
+        <f>6-G34</f>
+        <v/>
+      </c>
+      <c r="E37" s="19">
+        <f>6-G35</f>
+        <v/>
+      </c>
+      <c r="F37" s="19">
+        <f>6-G36</f>
+        <v/>
+      </c>
+      <c r="G37" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="C37" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="E37" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="19" t="n">
+      <c r="J37" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L37" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="G37" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="H37" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I37" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="J37" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K37" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="19" t="n">
-        <v>2</v>
-      </c>
       <c r="M37" s="19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" s="19" t="n">
         <v>3</v>
@@ -2186,7 +2184,7 @@
         <v>1</v>
       </c>
       <c r="P37" s="19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q37" s="19" t="n">
         <v>1</v>
@@ -2197,62 +2195,73 @@
       <c r="S37" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T37" s="20" t="n">
-        <v>1.94</v>
+      <c r="T37" s="20">
+        <f>SUM(H37:S37)+SUM(G32:G36)</f>
+        <v/>
+      </c>
+      <c r="U37" s="20">
+        <f>RANK(T37,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>Q8</t>
-        </is>
-      </c>
-      <c r="B38" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" s="19" t="n">
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="B38" s="19">
+        <f>6-H32</f>
+        <v/>
+      </c>
+      <c r="C38" s="19">
+        <f>6-H33</f>
+        <v/>
+      </c>
+      <c r="D38" s="19">
+        <f>6-H34</f>
+        <v/>
+      </c>
+      <c r="E38" s="19">
+        <f>6-H35</f>
+        <v/>
+      </c>
+      <c r="F38" s="19">
+        <f>6-H36</f>
+        <v/>
+      </c>
+      <c r="G38" s="19">
+        <f>6-H37</f>
+        <v/>
+      </c>
+      <c r="H38" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="N38" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="D38" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="E38" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F38" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="G38" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="H38" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="I38" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J38" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K38" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="L38" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="M38" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="N38" s="19" t="n">
-        <v>4</v>
-      </c>
       <c r="O38" s="19" t="n">
         <v>1</v>
       </c>
       <c r="P38" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q38" s="19" t="n">
         <v>1</v>
@@ -2263,63 +2272,75 @@
       <c r="S38" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T38" s="20" t="n">
-        <v>2.59</v>
+      <c r="T38" s="20">
+        <f>SUM(I38:S38)+SUM(H32:H37)</f>
+        <v/>
+      </c>
+      <c r="U38" s="20">
+        <f>RANK(T38,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>Q9</t>
-        </is>
-      </c>
-      <c r="B39" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C39" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="19" t="n">
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="B39" s="19">
+        <f>6-I32</f>
+        <v/>
+      </c>
+      <c r="C39" s="19">
+        <f>6-I33</f>
+        <v/>
+      </c>
+      <c r="D39" s="19">
+        <f>6-I34</f>
+        <v/>
+      </c>
+      <c r="E39" s="19">
+        <f>6-I35</f>
+        <v/>
+      </c>
+      <c r="F39" s="19">
+        <f>6-I36</f>
+        <v/>
+      </c>
+      <c r="G39" s="19">
+        <f>6-I37</f>
+        <v/>
+      </c>
+      <c r="H39" s="19">
+        <f>6-I38</f>
+        <v/>
+      </c>
+      <c r="I39" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L39" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M39" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="N39" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="F39" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I39" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K39" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="L39" s="19" t="n">
+      <c r="O39" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="M39" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N39" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="O39" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P39" s="19" t="n">
-        <v>1</v>
-      </c>
       <c r="Q39" s="19" t="n">
         <v>1</v>
       </c>
@@ -2329,47 +2350,60 @@
       <c r="S39" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T39" s="20" t="n">
-        <v>1.76</v>
+      <c r="T39" s="20">
+        <f>SUM(J39:S39)+SUM(I32:I38)</f>
+        <v/>
+      </c>
+      <c r="U39" s="20">
+        <f>RANK(T39,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="B40" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H40" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I40" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="J40" s="19" t="n">
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="B40" s="19">
+        <f>6-J32</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>6-J33</f>
+        <v/>
+      </c>
+      <c r="D40" s="19">
+        <f>6-J34</f>
+        <v/>
+      </c>
+      <c r="E40" s="19">
+        <f>6-J35</f>
+        <v/>
+      </c>
+      <c r="F40" s="19">
+        <f>6-J36</f>
+        <v/>
+      </c>
+      <c r="G40" s="19">
+        <f>6-J37</f>
+        <v/>
+      </c>
+      <c r="H40" s="19">
+        <f>6-J38</f>
+        <v/>
+      </c>
+      <c r="I40" s="19">
+        <f>6-J39</f>
+        <v/>
+      </c>
+      <c r="J40" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K40" s="19" t="n">
         <v>4</v>
-      </c>
-      <c r="K40" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
       </c>
       <c r="L40" s="19" t="n">
         <v>3</v>
@@ -2378,7 +2412,7 @@
         <v>1</v>
       </c>
       <c r="N40" s="19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O40" s="19" t="n">
         <v>1</v>
@@ -2395,51 +2429,65 @@
       <c r="S40" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T40" s="20" t="n">
-        <v>1.53</v>
+      <c r="T40" s="20">
+        <f>SUM(K40:S40)+SUM(J32:J39)</f>
+        <v/>
+      </c>
+      <c r="U40" s="20">
+        <f>RANK(T40,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>Q11</t>
-        </is>
-      </c>
-      <c r="B41" s="19" t="n">
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B41" s="19">
+        <f>6-K32</f>
+        <v/>
+      </c>
+      <c r="C41" s="19">
+        <f>6-K33</f>
+        <v/>
+      </c>
+      <c r="D41" s="19">
+        <f>6-K34</f>
+        <v/>
+      </c>
+      <c r="E41" s="19">
+        <f>6-K35</f>
+        <v/>
+      </c>
+      <c r="F41" s="19">
+        <f>6-K36</f>
+        <v/>
+      </c>
+      <c r="G41" s="19">
+        <f>6-K37</f>
+        <v/>
+      </c>
+      <c r="H41" s="19">
+        <f>6-K38</f>
+        <v/>
+      </c>
+      <c r="I41" s="19">
+        <f>6-K39</f>
+        <v/>
+      </c>
+      <c r="J41" s="19">
+        <f>6-K40</f>
+        <v/>
+      </c>
+      <c r="K41" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C41" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="D41" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E41" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="H41" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="I41" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="J41" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K41" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="L41" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="M41" s="19" t="n">
         <v>1</v>
       </c>
@@ -2450,7 +2498,7 @@
         <v>1</v>
       </c>
       <c r="P41" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q41" s="19" t="n">
         <v>1</v>
@@ -2461,56 +2509,71 @@
       <c r="S41" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T41" s="20" t="n">
-        <v>1.94</v>
+      <c r="T41" s="20">
+        <f>SUM(L41:S41)+SUM(K32:K40)</f>
+        <v/>
+      </c>
+      <c r="U41" s="20">
+        <f>RANK(T41,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="B42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="J42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L42" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M42" s="18" t="inlineStr">
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B42" s="19">
+        <f>6-L32</f>
+        <v/>
+      </c>
+      <c r="C42" s="19">
+        <f>6-L33</f>
+        <v/>
+      </c>
+      <c r="D42" s="19">
+        <f>6-L34</f>
+        <v/>
+      </c>
+      <c r="E42" s="19">
+        <f>6-L35</f>
+        <v/>
+      </c>
+      <c r="F42" s="19">
+        <f>6-L36</f>
+        <v/>
+      </c>
+      <c r="G42" s="19">
+        <f>6-L37</f>
+        <v/>
+      </c>
+      <c r="H42" s="19">
+        <f>6-L38</f>
+        <v/>
+      </c>
+      <c r="I42" s="19">
+        <f>6-L39</f>
+        <v/>
+      </c>
+      <c r="J42" s="19">
+        <f>6-L40</f>
+        <v/>
+      </c>
+      <c r="K42" s="19">
+        <f>6-L41</f>
+        <v/>
+      </c>
+      <c r="L42" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="M42" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="N42" s="19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O42" s="19" t="n">
         <v>1</v>
@@ -2527,57 +2590,73 @@
       <c r="S42" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T42" s="20" t="n">
-        <v>1.53</v>
+      <c r="T42" s="20">
+        <f>SUM(M42:S42)+SUM(L32:L41)</f>
+        <v/>
+      </c>
+      <c r="U42" s="20">
+        <f>RANK(T42,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="B43" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="F43" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="G43" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="H43" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="I43" s="19" t="n">
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B43" s="19">
+        <f>6-M32</f>
+        <v/>
+      </c>
+      <c r="C43" s="19">
+        <f>6-M33</f>
+        <v/>
+      </c>
+      <c r="D43" s="19">
+        <f>6-M34</f>
+        <v/>
+      </c>
+      <c r="E43" s="19">
+        <f>6-M35</f>
+        <v/>
+      </c>
+      <c r="F43" s="19">
+        <f>6-M36</f>
+        <v/>
+      </c>
+      <c r="G43" s="19">
+        <f>6-M37</f>
+        <v/>
+      </c>
+      <c r="H43" s="19">
+        <f>6-M38</f>
+        <v/>
+      </c>
+      <c r="I43" s="19">
+        <f>6-M39</f>
+        <v/>
+      </c>
+      <c r="J43" s="19">
+        <f>6-M40</f>
+        <v/>
+      </c>
+      <c r="K43" s="19">
+        <f>6-M41</f>
+        <v/>
+      </c>
+      <c r="L43" s="19">
+        <f>6-M42</f>
+        <v/>
+      </c>
+      <c r="M43" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N43" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J43" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K43" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L43" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M43" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="N43" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="O43" s="19" t="n">
         <v>1</v>
       </c>
@@ -2593,62 +2672,79 @@
       <c r="S43" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T43" s="20" t="n">
-        <v>1.88</v>
+      <c r="T43" s="20">
+        <f>SUM(N43:S43)+SUM(M32:M42)</f>
+        <v/>
+      </c>
+      <c r="U43" s="20">
+        <f>RANK(T43,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>Q14</t>
-        </is>
-      </c>
-      <c r="B44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N44" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O44" s="18" t="inlineStr">
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B44" s="19">
+        <f>6-N32</f>
+        <v/>
+      </c>
+      <c r="C44" s="19">
+        <f>6-N33</f>
+        <v/>
+      </c>
+      <c r="D44" s="19">
+        <f>6-N34</f>
+        <v/>
+      </c>
+      <c r="E44" s="19">
+        <f>6-N35</f>
+        <v/>
+      </c>
+      <c r="F44" s="19">
+        <f>6-N36</f>
+        <v/>
+      </c>
+      <c r="G44" s="19">
+        <f>6-N37</f>
+        <v/>
+      </c>
+      <c r="H44" s="19">
+        <f>6-N38</f>
+        <v/>
+      </c>
+      <c r="I44" s="19">
+        <f>6-N39</f>
+        <v/>
+      </c>
+      <c r="J44" s="19">
+        <f>6-N40</f>
+        <v/>
+      </c>
+      <c r="K44" s="19">
+        <f>6-N41</f>
+        <v/>
+      </c>
+      <c r="L44" s="19">
+        <f>6-N42</f>
+        <v/>
+      </c>
+      <c r="M44" s="19">
+        <f>6-N43</f>
+        <v/>
+      </c>
+      <c r="N44" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="O44" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="P44" s="19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Q44" s="19" t="n">
         <v>1</v>
@@ -2659,346 +2755,456 @@
       <c r="S44" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="T44" s="20" t="n">
-        <v>1.18</v>
+      <c r="T44" s="20">
+        <f>SUM(O44:S44)+SUM(N32:N43)</f>
+        <v/>
+      </c>
+      <c r="U44" s="20">
+        <f>RANK(T44,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>Q15</t>
-        </is>
-      </c>
-      <c r="B45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="E45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="G45" s="19" t="n">
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B45" s="19">
+        <f>6-O32</f>
+        <v/>
+      </c>
+      <c r="C45" s="19">
+        <f>6-O33</f>
+        <v/>
+      </c>
+      <c r="D45" s="19">
+        <f>6-O34</f>
+        <v/>
+      </c>
+      <c r="E45" s="19">
+        <f>6-O35</f>
+        <v/>
+      </c>
+      <c r="F45" s="19">
+        <f>6-O36</f>
+        <v/>
+      </c>
+      <c r="G45" s="19">
+        <f>6-O37</f>
+        <v/>
+      </c>
+      <c r="H45" s="19">
+        <f>6-O38</f>
+        <v/>
+      </c>
+      <c r="I45" s="19">
+        <f>6-O39</f>
+        <v/>
+      </c>
+      <c r="J45" s="19">
+        <f>6-O40</f>
+        <v/>
+      </c>
+      <c r="K45" s="19">
+        <f>6-O41</f>
+        <v/>
+      </c>
+      <c r="L45" s="19">
+        <f>6-O42</f>
+        <v/>
+      </c>
+      <c r="M45" s="19">
+        <f>6-O43</f>
+        <v/>
+      </c>
+      <c r="N45" s="19">
+        <f>6-O44</f>
+        <v/>
+      </c>
+      <c r="O45" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P45" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="H45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="I45" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J45" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K45" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="M45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="N45" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="O45" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="P45" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="Q45" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R45" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S45" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="T45" s="20" t="n">
-        <v>2.24</v>
+        <v>1</v>
+      </c>
+      <c r="T45" s="20">
+        <f>SUM(P45:S45)+SUM(O32:O44)</f>
+        <v/>
+      </c>
+      <c r="U45" s="20">
+        <f>RANK(T45,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>Q16</t>
-        </is>
-      </c>
-      <c r="B46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O46" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P46" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q46" s="18" t="inlineStr">
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B46" s="19">
+        <f>6-P32</f>
+        <v/>
+      </c>
+      <c r="C46" s="19">
+        <f>6-P33</f>
+        <v/>
+      </c>
+      <c r="D46" s="19">
+        <f>6-P34</f>
+        <v/>
+      </c>
+      <c r="E46" s="19">
+        <f>6-P35</f>
+        <v/>
+      </c>
+      <c r="F46" s="19">
+        <f>6-P36</f>
+        <v/>
+      </c>
+      <c r="G46" s="19">
+        <f>6-P37</f>
+        <v/>
+      </c>
+      <c r="H46" s="19">
+        <f>6-P38</f>
+        <v/>
+      </c>
+      <c r="I46" s="19">
+        <f>6-P39</f>
+        <v/>
+      </c>
+      <c r="J46" s="19">
+        <f>6-P40</f>
+        <v/>
+      </c>
+      <c r="K46" s="19">
+        <f>6-P41</f>
+        <v/>
+      </c>
+      <c r="L46" s="19">
+        <f>6-P42</f>
+        <v/>
+      </c>
+      <c r="M46" s="19">
+        <f>6-P43</f>
+        <v/>
+      </c>
+      <c r="N46" s="19">
+        <f>6-P44</f>
+        <v/>
+      </c>
+      <c r="O46" s="19">
+        <f>6-P45</f>
+        <v/>
+      </c>
+      <c r="P46" s="18" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
+      <c r="Q46" s="19" t="n">
+        <v>2</v>
+      </c>
       <c r="R46" s="19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="S46" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="T46" s="20" t="n">
-        <v>1.47</v>
+        <v>3</v>
+      </c>
+      <c r="T46" s="20">
+        <f>SUM(Q46:S46)+SUM(P32:P45)</f>
+        <v/>
+      </c>
+      <c r="U46" s="20">
+        <f>RANK(T46,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>Q17</t>
-        </is>
-      </c>
-      <c r="B47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O47" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P47" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q47" s="19" t="n">
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="B47" s="19">
+        <f>6-Q32</f>
+        <v/>
+      </c>
+      <c r="C47" s="19">
+        <f>6-Q33</f>
+        <v/>
+      </c>
+      <c r="D47" s="19">
+        <f>6-Q34</f>
+        <v/>
+      </c>
+      <c r="E47" s="19">
+        <f>6-Q35</f>
+        <v/>
+      </c>
+      <c r="F47" s="19">
+        <f>6-Q36</f>
+        <v/>
+      </c>
+      <c r="G47" s="19">
+        <f>6-Q37</f>
+        <v/>
+      </c>
+      <c r="H47" s="19">
+        <f>6-Q38</f>
+        <v/>
+      </c>
+      <c r="I47" s="19">
+        <f>6-Q39</f>
+        <v/>
+      </c>
+      <c r="J47" s="19">
+        <f>6-Q40</f>
+        <v/>
+      </c>
+      <c r="K47" s="19">
+        <f>6-Q41</f>
+        <v/>
+      </c>
+      <c r="L47" s="19">
+        <f>6-Q42</f>
+        <v/>
+      </c>
+      <c r="M47" s="19">
+        <f>6-Q43</f>
+        <v/>
+      </c>
+      <c r="N47" s="19">
+        <f>6-Q44</f>
+        <v/>
+      </c>
+      <c r="O47" s="19">
+        <f>6-Q45</f>
+        <v/>
+      </c>
+      <c r="P47" s="19">
+        <f>6-Q46</f>
+        <v/>
+      </c>
+      <c r="Q47" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R47" s="19" t="n">
         <v>5</v>
-      </c>
-      <c r="R47" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
       </c>
       <c r="S47" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="T47" s="20" t="n">
-        <v>1.47</v>
+      <c r="T47" s="20">
+        <f>SUM(R47:S47)+SUM(Q32:Q46)</f>
+        <v/>
+      </c>
+      <c r="U47" s="20">
+        <f>RANK(T47,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>Q18</t>
-        </is>
-      </c>
-      <c r="B48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="H48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="L48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="M48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="O48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="P48" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q48" s="19" t="n">
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="B48" s="19">
+        <f>6-R32</f>
+        <v/>
+      </c>
+      <c r="C48" s="19">
+        <f>6-R33</f>
+        <v/>
+      </c>
+      <c r="D48" s="19">
+        <f>6-R34</f>
+        <v/>
+      </c>
+      <c r="E48" s="19">
+        <f>6-R35</f>
+        <v/>
+      </c>
+      <c r="F48" s="19">
+        <f>6-R36</f>
+        <v/>
+      </c>
+      <c r="G48" s="19">
+        <f>6-R37</f>
+        <v/>
+      </c>
+      <c r="H48" s="19">
+        <f>6-R38</f>
+        <v/>
+      </c>
+      <c r="I48" s="19">
+        <f>6-R39</f>
+        <v/>
+      </c>
+      <c r="J48" s="19">
+        <f>6-R40</f>
+        <v/>
+      </c>
+      <c r="K48" s="19">
+        <f>6-R41</f>
+        <v/>
+      </c>
+      <c r="L48" s="19">
+        <f>6-R42</f>
+        <v/>
+      </c>
+      <c r="M48" s="19">
+        <f>6-R43</f>
+        <v/>
+      </c>
+      <c r="N48" s="19">
+        <f>6-R44</f>
+        <v/>
+      </c>
+      <c r="O48" s="19">
+        <f>6-R45</f>
+        <v/>
+      </c>
+      <c r="P48" s="19">
+        <f>6-R46</f>
+        <v/>
+      </c>
+      <c r="Q48" s="19">
+        <f>6-R47</f>
+        <v/>
+      </c>
+      <c r="R48" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S48" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="R48" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="S48" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T48" s="20" t="n">
-        <v>1.47</v>
+      <c r="T48" s="20">
+        <f>SUM(S48:S48)+SUM(R32:R47)</f>
+        <v/>
+      </c>
+      <c r="U48" s="20">
+        <f>RANK(T48,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
         <is>
-          <t>Avg</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="C49" s="20" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="D49" s="20" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="E49" s="20" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="F49" s="20" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="G49" s="20" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="H49" s="20" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="I49" s="20" t="n">
-        <v>2.59</v>
-      </c>
-      <c r="J49" s="20" t="n">
-        <v>1.76</v>
-      </c>
-      <c r="K49" s="20" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="L49" s="20" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="M49" s="20" t="n">
-        <v>1.53</v>
-      </c>
-      <c r="N49" s="20" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="O49" s="20" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="P49" s="20" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="Q49" s="20" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="R49" s="20" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="S49" s="20" t="n">
-        <v>1.47</v>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="B49" s="19">
+        <f>6-S32</f>
+        <v/>
+      </c>
+      <c r="C49" s="19">
+        <f>6-S33</f>
+        <v/>
+      </c>
+      <c r="D49" s="19">
+        <f>6-S34</f>
+        <v/>
+      </c>
+      <c r="E49" s="19">
+        <f>6-S35</f>
+        <v/>
+      </c>
+      <c r="F49" s="19">
+        <f>6-S36</f>
+        <v/>
+      </c>
+      <c r="G49" s="19">
+        <f>6-S37</f>
+        <v/>
+      </c>
+      <c r="H49" s="19">
+        <f>6-S38</f>
+        <v/>
+      </c>
+      <c r="I49" s="19">
+        <f>6-S39</f>
+        <v/>
+      </c>
+      <c r="J49" s="19">
+        <f>6-S40</f>
+        <v/>
+      </c>
+      <c r="K49" s="19">
+        <f>6-S41</f>
+        <v/>
+      </c>
+      <c r="L49" s="19">
+        <f>6-S42</f>
+        <v/>
+      </c>
+      <c r="M49" s="19">
+        <f>6-S43</f>
+        <v/>
+      </c>
+      <c r="N49" s="19">
+        <f>6-S44</f>
+        <v/>
+      </c>
+      <c r="O49" s="19">
+        <f>6-S45</f>
+        <v/>
+      </c>
+      <c r="P49" s="19">
+        <f>6-S46</f>
+        <v/>
+      </c>
+      <c r="Q49" s="19">
+        <f>6-S47</f>
+        <v/>
+      </c>
+      <c r="R49" s="19">
+        <f>6-S48</f>
+        <v/>
+      </c>
+      <c r="S49" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T49" s="20">
+        <f>SUM(S32:S48)</f>
+        <v/>
+      </c>
+      <c r="U49" s="20">
+        <f>RANK(T49,T32:T49,0)</f>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="15" t="inlineStr">
         <is>
-          <t>Notable overlaps (score 4-5)</t>
+          <t>Notable primary overlaps (score 4-5)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
         <is>
-          <t>Pair</t>
+          <t>Direction</t>
         </is>
       </c>
       <c r="B52" s="17" t="inlineStr">
@@ -3008,267 +3214,323 @@
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
+          <t>Reverse (auto)</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
           <t>Why</t>
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="45" customHeight="1">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t>Q1 &lt;-&gt; Q7</t>
+          <t>Q1 -&gt; Q7</t>
         </is>
       </c>
       <c r="B53" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C53" s="12" t="inlineStr">
+      <c r="C53" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>Near-duplicate: both ask about having a clearly defined career-path structure.</t>
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="45" customHeight="1">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>Q3 &lt;-&gt; Q5</t>
+          <t>Q3 -&gt; Q5</t>
         </is>
       </c>
       <c r="B54" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C54" s="14" t="inlineStr">
+      <c r="C54" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>Both are about how promotion decisions are made (clarity vs. fairness/consistency).</t>
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="45" customHeight="1">
       <c r="A55" s="12" t="inlineStr">
         <is>
-          <t>Q6 &lt;-&gt; Q8</t>
+          <t>Q6 -&gt; Q8</t>
         </is>
       </c>
       <c r="B55" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C55" s="12" t="inlineStr">
+      <c r="C55" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="12" t="inlineStr">
         <is>
           <t>Two sides of the same coin: desired fix vs. the pain point it would fix.</t>
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="45" customHeight="1">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>Q8 &lt;-&gt; Q12</t>
+          <t>Q8 -&gt; Q12</t>
         </is>
       </c>
       <c r="B56" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C56" s="14" t="inlineStr">
+      <c r="C56" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>Q12 is an explicit follow-up to the biggest-challenge question (Q8).</t>
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="45" customHeight="1">
       <c r="A57" s="12" t="inlineStr">
         <is>
-          <t>Q16 &lt;-&gt; Q17</t>
+          <t>Q16 -&gt; Q17</t>
         </is>
       </c>
       <c r="B57" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C57" s="12" t="inlineStr">
+      <c r="C57" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" s="12" t="inlineStr">
         <is>
           <t>Both measure awareness/understanding of the 2030 EBITDA target.</t>
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="45" customHeight="1">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>Q1 &lt;-&gt; Q3</t>
+          <t>Q1 -&gt; Q3</t>
         </is>
       </c>
       <c r="B58" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C58" s="14" t="inlineStr">
+      <c r="C58" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>Both measure clarity of the advancement structure (path vs. promotion criteria).</t>
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="45" customHeight="1">
       <c r="A59" s="12" t="inlineStr">
         <is>
-          <t>Q2 &lt;-&gt; Q4</t>
+          <t>Q2 -&gt; Q4</t>
         </is>
       </c>
       <c r="B59" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C59" s="12" t="inlineStr">
+      <c r="C59" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="12" t="inlineStr">
         <is>
           <t>Both concern availability/quality of the same L&amp;D resources (awareness vs. accessibility &amp; adequacy).</t>
         </is>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="45" customHeight="1">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>Q3 &lt;-&gt; Q7</t>
+          <t>Q3 -&gt; Q7</t>
         </is>
       </c>
       <c r="B60" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C60" s="14" t="inlineStr">
+      <c r="C60" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>Both about structural clarity of career advancement.</t>
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="45" customHeight="1">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t>Q3 &lt;-&gt; Q8</t>
+          <t>Q3 -&gt; Q8</t>
         </is>
       </c>
       <c r="B61" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C61" s="12" t="inlineStr">
+      <c r="C61" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
         <is>
           <t>The challenge MCQ explicitly includes 'promotion criteria are unclear' as an option.</t>
         </is>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="45" customHeight="1">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>Q4 &lt;-&gt; Q9</t>
+          <t>Q4 -&gt; Q9</t>
         </is>
       </c>
       <c r="B62" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C62" s="14" t="inlineStr">
+      <c r="C62" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
         <is>
           <t>Both measure sufficiency of development support (general adequacy vs. technical skill currency).</t>
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="45" customHeight="1">
       <c r="A63" s="12" t="inlineStr">
         <is>
-          <t>Q6 &lt;-&gt; Q15</t>
+          <t>Q6 -&gt; Q15</t>
         </is>
       </c>
       <c r="B63" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C63" s="12" t="inlineStr">
+      <c r="C63" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
         <is>
           <t>Same intent (what would help), different format: closed MCQ vs. open catch-all.</t>
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="45" customHeight="1">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>Q8 &lt;-&gt; Q13</t>
+          <t>Q8 -&gt; Q13</t>
         </is>
       </c>
       <c r="B64" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C64" s="14" t="inlineStr">
+      <c r="C64" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
         <is>
           <t>Root cause is asked about the same 'issue' identified by the challenge question (Q8).</t>
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="45" customHeight="1">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t>Q9 &lt;-&gt; Q10</t>
+          <t>Q9 -&gt; Q10</t>
         </is>
       </c>
       <c r="B65" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C65" s="12" t="inlineStr">
+      <c r="C65" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="12" t="inlineStr">
         <is>
           <t>Both are Ungku's technical-exposure sub-questions (skill currency vs. stretch assignments).</t>
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="45" customHeight="1">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>Q12 &lt;-&gt; Q13</t>
+          <t>Q12 -&gt; Q13</t>
         </is>
       </c>
       <c r="B66" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C66" s="14" t="inlineStr">
+      <c r="C66" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
         <is>
           <t>Paired diagnostic questions about the same issue: severity and root cause.</t>
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="45" customHeight="1">
       <c r="A67" s="12" t="inlineStr">
         <is>
-          <t>Q14 &lt;-&gt; Q15</t>
+          <t>Q14 -&gt; Q15</t>
         </is>
       </c>
       <c r="B67" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C67" s="12" t="inlineStr">
+      <c r="C67" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" s="12" t="inlineStr">
         <is>
           <t>Mark Turner's retention/development pair — both about staying/leaving sentiment.</t>
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="45" customHeight="1">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>Q16 &lt;-&gt; Q18</t>
+          <t>Q16 -&gt; Q18</t>
         </is>
       </c>
       <c r="B68" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C68" s="14" t="inlineStr">
+      <c r="C68" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>Same EBITDA-target topic cluster (awareness vs. barriers).</t>
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="45" customHeight="1">
       <c r="A69" s="12" t="inlineStr">
         <is>
-          <t>Q17 &lt;-&gt; Q18</t>
+          <t>Q17 -&gt; Q18</t>
         </is>
       </c>
       <c r="B69" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="C69" s="12" t="inlineStr">
+      <c r="C69" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" s="12" t="inlineStr">
         <is>
           <t>Same EBITDA-target topic cluster (role contribution vs. barriers).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B31:S48">
+  <conditionalFormatting sqref="B32:S49">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="1"/>

</xml_diff>